<commit_message>
Admin: Adiciona suporte a coluna de Status no upload de histórico do ranking
</commit_message>
<xml_diff>
--- a/static/planilha_historico.xlsx
+++ b/static/planilha_historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,11 @@
           <t>Rodada</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -473,6 +478,11 @@
       <c r="F2" t="n">
         <v>1</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>finalizado</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -489,7 +499,7 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -498,6 +508,11 @@
       </c>
       <c r="F3" t="n">
         <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>pendente</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>